<commit_message>
Fix startup window behavior and update mold catalog tests
</commit_message>
<xml_diff>
--- a/data/Moldes.xlsx
+++ b/data/Moldes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\procesos.CAZEL\Desktop\BECARIO PROCESOS\AUTOMATIZACIÓN DE PARÁMETROS\AutomatizacionParametros_v3.0\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F635EC9-9217-4CB5-B9FD-6595153AD900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FAE49A-6C81-4E87-9567-E3551189FA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11333" uniqueCount="6199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11543" uniqueCount="6220">
   <si>
     <t>Molde</t>
   </si>
@@ -18621,6 +18621,69 @@
   </si>
   <si>
     <t>MAGNA DECOPLAS</t>
+  </si>
+  <si>
+    <t>LEAR</t>
+  </si>
+  <si>
+    <t>PSW</t>
+  </si>
+  <si>
+    <t>PLASMAN</t>
+  </si>
+  <si>
+    <t>VALEO</t>
+  </si>
+  <si>
+    <t>OP MOBILITY LIGHTING</t>
+  </si>
+  <si>
+    <t>FLEX</t>
+  </si>
+  <si>
+    <t>ZKW</t>
+  </si>
+  <si>
+    <t>MITZU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FREUDENBERG </t>
+  </si>
+  <si>
+    <t>DRAEXLMAIER</t>
+  </si>
+  <si>
+    <t>KTM</t>
+  </si>
+  <si>
+    <t>PTM</t>
+  </si>
+  <si>
+    <t>FUJIKURA</t>
+  </si>
+  <si>
+    <t>YANFENG</t>
+  </si>
+  <si>
+    <t>JANESVILLE</t>
+  </si>
+  <si>
+    <t>DIEHL</t>
+  </si>
+  <si>
+    <t>CELESTICA</t>
+  </si>
+  <si>
+    <t>KOBLENZ</t>
+  </si>
+  <si>
+    <t>REHAU</t>
+  </si>
+  <si>
+    <t>KOSTAL</t>
+  </si>
+  <si>
+    <t>KASAI MEXICANA</t>
   </si>
 </sst>
 </file>
@@ -20020,7 +20083,7 @@
         <v>141</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>143</v>
@@ -20031,16 +20094,14 @@
       <c r="E51" s="3">
         <v>56</v>
       </c>
-      <c r="F51" s="2" t="s">
-        <v>149</v>
-      </c>
+      <c r="F51" s="2"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>141</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>146</v>
@@ -20051,22 +20112,20 @@
       <c r="E52" s="3">
         <v>56</v>
       </c>
-      <c r="F52" s="2" t="s">
-        <v>149</v>
-      </c>
+      <c r="F52" s="2"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>141</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E53" s="3">
         <v>56</v>
@@ -20080,13 +20139,13 @@
         <v>141</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>146</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="E54" s="3">
         <v>56</v>
@@ -20100,43 +20159,47 @@
         <v>141</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="E55" s="3">
         <v>56</v>
       </c>
-      <c r="F55" s="2"/>
+      <c r="F55" s="2" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>141</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>146</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="E56" s="3">
         <v>56</v>
       </c>
-      <c r="F56" s="2"/>
+      <c r="F56" s="2" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>155</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>157</v>
@@ -20147,16 +20210,14 @@
       <c r="E57" s="3">
         <v>44</v>
       </c>
-      <c r="F57" s="2" t="s">
-        <v>149</v>
-      </c>
+      <c r="F57" s="2"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>155</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>160</v>
@@ -20167,22 +20228,20 @@
       <c r="E58" s="3">
         <v>44</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>149</v>
-      </c>
+      <c r="F58" s="2"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>155</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>157</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="E59" s="3">
         <v>44</v>
@@ -20196,13 +20255,13 @@
         <v>155</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>160</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E60" s="3">
         <v>44</v>
@@ -20216,43 +20275,47 @@
         <v>155</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>157</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="E61" s="3">
         <v>44</v>
       </c>
-      <c r="F61" s="2"/>
+      <c r="F61" s="2" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>155</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>160</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E62" s="3">
         <v>44</v>
       </c>
-      <c r="F62" s="2"/>
+      <c r="F62" s="2" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>170</v>
@@ -20263,22 +20326,20 @@
       <c r="E63" s="3">
         <v>51</v>
       </c>
-      <c r="F63" s="2" t="s">
-        <v>149</v>
-      </c>
+      <c r="F63" s="2"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>170</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E64" s="3">
         <v>51</v>
@@ -20292,18 +20353,20 @@
         <v>168</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>170</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E65" s="3">
         <v>51</v>
       </c>
-      <c r="F65" s="2"/>
+      <c r="F65" s="2" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
@@ -20921,7 +20984,9 @@
       <c r="E98" s="3">
         <v>21</v>
       </c>
-      <c r="F98" s="2"/>
+      <c r="F98" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
@@ -20939,7 +21004,9 @@
       <c r="E99" s="3">
         <v>25</v>
       </c>
-      <c r="F99" s="2"/>
+      <c r="F99" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
@@ -20957,7 +21024,9 @@
       <c r="E100" s="3">
         <v>36</v>
       </c>
-      <c r="F100" s="2"/>
+      <c r="F100" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
@@ -20975,7 +21044,9 @@
       <c r="E101" s="3">
         <v>21</v>
       </c>
-      <c r="F101" s="2"/>
+      <c r="F101" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
@@ -20993,7 +21064,9 @@
       <c r="E102" s="3">
         <v>21</v>
       </c>
-      <c r="F102" s="2"/>
+      <c r="F102" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
@@ -21011,7 +21084,9 @@
       <c r="E103" s="3">
         <v>21</v>
       </c>
-      <c r="F103" s="2"/>
+      <c r="F103" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
@@ -21029,7 +21104,9 @@
       <c r="E104" s="3">
         <v>19</v>
       </c>
-      <c r="F104" s="2"/>
+      <c r="F104" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
@@ -21207,7 +21284,9 @@
       <c r="E113" s="3">
         <v>69</v>
       </c>
-      <c r="F113" s="2"/>
+      <c r="F113" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
@@ -21225,7 +21304,9 @@
       <c r="E114" s="3">
         <v>69</v>
       </c>
-      <c r="F114" s="2"/>
+      <c r="F114" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
@@ -21243,7 +21324,9 @@
       <c r="E115" s="3">
         <v>69</v>
       </c>
-      <c r="F115" s="2"/>
+      <c r="F115" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
@@ -21397,7 +21480,9 @@
       <c r="E123" s="3">
         <v>22</v>
       </c>
-      <c r="F123" s="2"/>
+      <c r="F123" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
@@ -21415,7 +21500,9 @@
       <c r="E124" s="3">
         <v>22</v>
       </c>
-      <c r="F124" s="2"/>
+      <c r="F124" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
@@ -21433,7 +21520,9 @@
       <c r="E125" s="3">
         <v>22</v>
       </c>
-      <c r="F125" s="2"/>
+      <c r="F125" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
@@ -21451,7 +21540,9 @@
       <c r="E126" s="3">
         <v>22</v>
       </c>
-      <c r="F126" s="2"/>
+      <c r="F126" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
@@ -21469,7 +21560,9 @@
       <c r="E127" s="3">
         <v>60</v>
       </c>
-      <c r="F127" s="2"/>
+      <c r="F127" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
@@ -21487,7 +21580,9 @@
       <c r="E128" s="3">
         <v>78</v>
       </c>
-      <c r="F128" s="2"/>
+      <c r="F128" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
@@ -21505,7 +21600,9 @@
       <c r="E129" s="3">
         <v>78</v>
       </c>
-      <c r="F129" s="2"/>
+      <c r="F129" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
@@ -21523,34 +21620,34 @@
       <c r="E130" s="3">
         <v>24</v>
       </c>
-      <c r="F130" s="2"/>
+      <c r="F130" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>356</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="E131" s="3">
-        <v>28</v>
-      </c>
-      <c r="F131" s="2" t="s">
-        <v>10</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="F131" s="2"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>356</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>358</v>
@@ -21570,16 +21667,16 @@
         <v>356</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E133" s="3">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F133" s="2" t="s">
         <v>10</v>
@@ -21590,18 +21687,20 @@
         <v>356</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="E134" s="3">
         <v>25</v>
       </c>
-      <c r="F134" s="2"/>
+      <c r="F134" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
@@ -21619,7 +21718,9 @@
       <c r="E135" s="3">
         <v>60</v>
       </c>
-      <c r="F135" s="2"/>
+      <c r="F135" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
@@ -21637,7 +21738,9 @@
       <c r="E136" s="3">
         <v>60</v>
       </c>
-      <c r="F136" s="2"/>
+      <c r="F136" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
@@ -21655,7 +21758,9 @@
       <c r="E137" s="3">
         <v>180</v>
       </c>
-      <c r="F137" s="2"/>
+      <c r="F137" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
@@ -21673,7 +21778,9 @@
       <c r="E138" s="3">
         <v>180</v>
       </c>
-      <c r="F138" s="2"/>
+      <c r="F138" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
@@ -21696,38 +21803,38 @@
         <v>384</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>386</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="E140" s="3">
         <v>60</v>
       </c>
-      <c r="F140" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F140" s="2"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>384</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C141" s="2" t="s">
         <v>386</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E141" s="3">
         <v>60</v>
       </c>
-      <c r="F141" s="2"/>
+      <c r="F141" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
@@ -21745,7 +21852,9 @@
       <c r="E142" s="3">
         <v>113</v>
       </c>
-      <c r="F142" s="2"/>
+      <c r="F142" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
@@ -21852,33 +21961,31 @@
         <v>412</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E148" s="3">
         <v>40</v>
       </c>
-      <c r="F148" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F148" s="2"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>412</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E149" s="3">
         <v>40</v>
@@ -21892,18 +21999,20 @@
         <v>412</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="E150" s="3">
         <v>40</v>
       </c>
-      <c r="F150" s="2"/>
+      <c r="F150" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
@@ -23394,7 +23503,7 @@
         <v>628</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>640</v>
+        <v>629</v>
       </c>
       <c r="C227" s="2" t="s">
         <v>630</v>
@@ -23405,22 +23514,20 @@
       <c r="E227" s="3">
         <v>25</v>
       </c>
-      <c r="F227" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F227" s="2"/>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
         <v>628</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="E228" s="3">
         <v>25</v>
@@ -23438,7 +23545,7 @@
         <v>633</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E229" s="3">
         <v>25</v>
@@ -23450,13 +23557,13 @@
         <v>628</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="E230" s="3">
         <v>25</v>
@@ -23468,7 +23575,7 @@
         <v>628</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="C231" s="2" t="s">
         <v>637</v>
@@ -23486,52 +23593,54 @@
         <v>628</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>637</v>
+        <v>630</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>638</v>
+        <v>631</v>
       </c>
       <c r="E232" s="3">
         <v>25</v>
       </c>
-      <c r="F232" s="2"/>
+      <c r="F232" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="233" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
         <v>641</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="D233" s="2"/>
       <c r="E233" s="3">
-        <v>69</v>
-      </c>
-      <c r="F233" s="2" t="s">
-        <v>178</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="F233" s="2"/>
     </row>
     <row r="234" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>641</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="D234" s="2"/>
       <c r="E234" s="3">
-        <v>68</v>
-      </c>
-      <c r="F234" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="F234" s="2" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
@@ -23686,76 +23795,76 @@
         <v>665</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="C243" s="2" t="s">
         <v>673</v>
       </c>
       <c r="D243" s="2" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="E243" s="3">
         <v>38</v>
       </c>
-      <c r="F243" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F243" s="2"/>
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
         <v>665</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="C244" s="2" t="s">
         <v>667</v>
       </c>
       <c r="D244" s="2" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="E244" s="3">
         <v>38</v>
       </c>
-      <c r="F244" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F244" s="2"/>
     </row>
     <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="2" t="s">
         <v>665</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="C245" s="2" t="s">
         <v>673</v>
       </c>
       <c r="D245" s="2" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="E245" s="3">
         <v>38</v>
       </c>
-      <c r="F245" s="2"/>
+      <c r="F245" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" s="2" t="s">
         <v>665</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>667</v>
       </c>
       <c r="D246" s="2" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="E246" s="3">
         <v>38</v>
       </c>
-      <c r="F246" s="2"/>
+      <c r="F246" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" s="2" t="s">
@@ -23906,152 +24015,152 @@
         <v>681</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="C255" s="2" t="s">
         <v>673</v>
       </c>
       <c r="D255" s="2" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="E255" s="3">
         <v>36</v>
       </c>
-      <c r="F255" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F255" s="2"/>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="C256" s="2" t="s">
         <v>686</v>
       </c>
       <c r="D256" s="2" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="E256" s="3">
         <v>36</v>
       </c>
-      <c r="F256" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F256" s="2"/>
     </row>
     <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="C257" s="2" t="s">
         <v>673</v>
       </c>
       <c r="D257" s="2" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="E257" s="3">
         <v>36</v>
       </c>
-      <c r="F257" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F257" s="2"/>
     </row>
     <row r="258" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>712</v>
+        <v>704</v>
       </c>
       <c r="C258" s="2" t="s">
         <v>683</v>
       </c>
       <c r="D258" s="2" t="s">
-        <v>713</v>
+        <v>705</v>
       </c>
       <c r="E258" s="3">
         <v>36</v>
       </c>
-      <c r="F258" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F258" s="2"/>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="C259" s="2" t="s">
         <v>673</v>
       </c>
       <c r="D259" s="2" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="E259" s="3">
         <v>36</v>
       </c>
-      <c r="F259" s="2"/>
+      <c r="F259" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="C260" s="2" t="s">
         <v>686</v>
       </c>
       <c r="D260" s="2" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="E260" s="3">
         <v>36</v>
       </c>
-      <c r="F260" s="2"/>
+      <c r="F260" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="C261" s="2" t="s">
         <v>673</v>
       </c>
       <c r="D261" s="2" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="E261" s="3">
         <v>36</v>
       </c>
-      <c r="F261" s="2"/>
+      <c r="F261" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A262" s="2" t="s">
         <v>681</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="C262" s="2" t="s">
         <v>683</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="E262" s="3">
         <v>36</v>
       </c>
-      <c r="F262" s="2"/>
+      <c r="F262" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
@@ -24209,7 +24318,9 @@
       <c r="E270" s="3">
         <v>64</v>
       </c>
-      <c r="F270" s="2"/>
+      <c r="F270" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="271" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
@@ -24227,7 +24338,9 @@
       <c r="E271" s="3">
         <v>64</v>
       </c>
-      <c r="F271" s="2"/>
+      <c r="F271" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
@@ -24365,7 +24478,9 @@
       <c r="E278" s="3">
         <v>53</v>
       </c>
-      <c r="F278" s="2"/>
+      <c r="F278" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="279" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
@@ -24383,7 +24498,9 @@
       <c r="E279" s="3">
         <v>53</v>
       </c>
-      <c r="F279" s="2"/>
+      <c r="F279" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
@@ -24401,7 +24518,9 @@
       <c r="E280" s="3">
         <v>53</v>
       </c>
-      <c r="F280" s="2"/>
+      <c r="F280" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
@@ -24419,7 +24538,9 @@
       <c r="E281" s="3">
         <v>53</v>
       </c>
-      <c r="F281" s="2"/>
+      <c r="F281" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
@@ -24477,7 +24598,9 @@
       <c r="E284" s="3">
         <v>56</v>
       </c>
-      <c r="F284" s="2"/>
+      <c r="F284" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="285" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
@@ -24495,7 +24618,9 @@
       <c r="E285" s="3">
         <v>56</v>
       </c>
-      <c r="F285" s="2"/>
+      <c r="F285" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="286" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A286" s="2" t="s">
@@ -24677,7 +24802,9 @@
       <c r="E295" s="3">
         <v>55</v>
       </c>
-      <c r="F295" s="2"/>
+      <c r="F295" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
@@ -24695,7 +24822,9 @@
       <c r="E296" s="3">
         <v>55</v>
       </c>
-      <c r="F296" s="2"/>
+      <c r="F296" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
@@ -24711,7 +24840,9 @@
       <c r="E297" s="3">
         <v>33</v>
       </c>
-      <c r="F297" s="2"/>
+      <c r="F297" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
@@ -24727,7 +24858,9 @@
       <c r="E298" s="3">
         <v>33</v>
       </c>
-      <c r="F298" s="2"/>
+      <c r="F298" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
@@ -24786,33 +24919,31 @@
         <v>815</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="C302" s="2" t="s">
         <v>817</v>
       </c>
       <c r="D302" s="2" t="s">
-        <v>818</v>
+        <v>823</v>
       </c>
       <c r="E302" s="3">
         <v>25</v>
       </c>
-      <c r="F302" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F302" s="2"/>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
         <v>815</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="D303" s="2" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="E303" s="3">
         <v>25</v>
@@ -24826,18 +24957,20 @@
         <v>815</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="D304" s="2" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="E304" s="3">
         <v>25</v>
       </c>
-      <c r="F304" s="2"/>
+      <c r="F304" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
@@ -25015,7 +25148,9 @@
       <c r="E313" s="3">
         <v>55</v>
       </c>
-      <c r="F313" s="2"/>
+      <c r="F313" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
@@ -25033,7 +25168,9 @@
       <c r="E314" s="3">
         <v>55</v>
       </c>
-      <c r="F314" s="2"/>
+      <c r="F314" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A315" s="2" t="s">
@@ -25051,7 +25188,9 @@
       <c r="E315" s="3">
         <v>55</v>
       </c>
-      <c r="F315" s="2"/>
+      <c r="F315" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A316" s="2" t="s">
@@ -25069,7 +25208,9 @@
       <c r="E316" s="3">
         <v>55</v>
       </c>
-      <c r="F316" s="2"/>
+      <c r="F316" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
@@ -25573,7 +25714,9 @@
       <c r="E342" s="3">
         <v>61</v>
       </c>
-      <c r="F342" s="2"/>
+      <c r="F342" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
@@ -25589,7 +25732,9 @@
       <c r="E343" s="3">
         <v>60</v>
       </c>
-      <c r="F343" s="2"/>
+      <c r="F343" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
@@ -25605,7 +25750,9 @@
       <c r="E344" s="3">
         <v>61</v>
       </c>
-      <c r="F344" s="2"/>
+      <c r="F344" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
@@ -25621,7 +25768,9 @@
       <c r="E345" s="3">
         <v>60</v>
       </c>
-      <c r="F345" s="2"/>
+      <c r="F345" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
@@ -26391,7 +26540,9 @@
       <c r="E385" s="3">
         <v>24</v>
       </c>
-      <c r="F385" s="2"/>
+      <c r="F385" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A386" s="2" t="s">
@@ -26409,7 +26560,9 @@
       <c r="E386" s="3">
         <v>24</v>
       </c>
-      <c r="F386" s="2"/>
+      <c r="F386" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A387" s="2" t="s">
@@ -26427,7 +26580,9 @@
       <c r="E387" s="3">
         <v>24</v>
       </c>
-      <c r="F387" s="2"/>
+      <c r="F387" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A388" s="2" t="s">
@@ -26445,7 +26600,9 @@
       <c r="E388" s="3">
         <v>24</v>
       </c>
-      <c r="F388" s="2"/>
+      <c r="F388" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A389" s="2" t="s">
@@ -26479,7 +26636,9 @@
       <c r="E390" s="3">
         <v>32</v>
       </c>
-      <c r="F390" s="2"/>
+      <c r="F390" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A391" s="2" t="s">
@@ -26497,7 +26656,9 @@
       <c r="E391" s="3">
         <v>32</v>
       </c>
-      <c r="F391" s="2"/>
+      <c r="F391" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A392" s="2" t="s">
@@ -26515,7 +26676,9 @@
       <c r="E392" s="3">
         <v>32</v>
       </c>
-      <c r="F392" s="2"/>
+      <c r="F392" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A393" s="2" t="s">
@@ -26533,7 +26696,9 @@
       <c r="E393" s="3">
         <v>32</v>
       </c>
-      <c r="F393" s="2"/>
+      <c r="F393" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A394" s="2" t="s">
@@ -26611,7 +26776,9 @@
       <c r="E397" s="3">
         <v>40</v>
       </c>
-      <c r="F397" s="2"/>
+      <c r="F397" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="398" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A398" s="2" t="s">
@@ -26629,7 +26796,9 @@
       <c r="E398" s="3">
         <v>40</v>
       </c>
-      <c r="F398" s="2"/>
+      <c r="F398" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A399" s="2" t="s">
@@ -27223,7 +27392,9 @@
       <c r="E430" s="3">
         <v>30</v>
       </c>
-      <c r="F430" s="2"/>
+      <c r="F430" s="2" t="s">
+        <v>6208</v>
+      </c>
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A431" s="2" t="s">
@@ -27401,7 +27572,9 @@
       <c r="E439" s="3">
         <v>60</v>
       </c>
-      <c r="F439" s="2"/>
+      <c r="F439" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A440" s="2" t="s">
@@ -27419,7 +27592,9 @@
       <c r="E440" s="3">
         <v>55</v>
       </c>
-      <c r="F440" s="2"/>
+      <c r="F440" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="441" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A441" s="2" t="s">
@@ -27846,99 +28021,91 @@
         <v>1211</v>
       </c>
       <c r="B462" s="2" t="s">
-        <v>1212</v>
+        <v>1229</v>
       </c>
       <c r="C462" s="2" t="s">
-        <v>1213</v>
+        <v>1221</v>
       </c>
       <c r="D462" s="2" t="s">
-        <v>1214</v>
+        <v>1222</v>
       </c>
       <c r="E462" s="3">
         <v>55</v>
       </c>
-      <c r="F462" s="2" t="s">
-        <v>398</v>
-      </c>
+      <c r="F462" s="2"/>
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A463" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B463" s="2" t="s">
-        <v>1215</v>
+        <v>1230</v>
       </c>
       <c r="C463" s="2" t="s">
-        <v>1216</v>
+        <v>1221</v>
       </c>
       <c r="D463" s="2" t="s">
-        <v>1217</v>
+        <v>1224</v>
       </c>
       <c r="E463" s="3">
         <v>55</v>
       </c>
-      <c r="F463" s="2" t="s">
-        <v>398</v>
-      </c>
+      <c r="F463" s="2"/>
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A464" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B464" s="2" t="s">
-        <v>1218</v>
+        <v>1231</v>
       </c>
       <c r="C464" s="2" t="s">
-        <v>1213</v>
+        <v>1221</v>
       </c>
       <c r="D464" s="2" t="s">
-        <v>1219</v>
+        <v>1226</v>
       </c>
       <c r="E464" s="3">
         <v>55</v>
       </c>
-      <c r="F464" s="2" t="s">
-        <v>398</v>
-      </c>
+      <c r="F464" s="2"/>
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A465" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B465" s="2" t="s">
-        <v>1220</v>
+        <v>1232</v>
       </c>
       <c r="C465" s="2" t="s">
         <v>1221</v>
       </c>
       <c r="D465" s="2" t="s">
-        <v>1222</v>
+        <v>1228</v>
       </c>
       <c r="E465" s="3">
         <v>55</v>
       </c>
-      <c r="F465" s="2" t="s">
-        <v>454</v>
-      </c>
+      <c r="F465" s="2"/>
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A466" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B466" s="2" t="s">
-        <v>1223</v>
+        <v>1212</v>
       </c>
       <c r="C466" s="2" t="s">
-        <v>1221</v>
+        <v>1213</v>
       </c>
       <c r="D466" s="2" t="s">
-        <v>1224</v>
+        <v>1214</v>
       </c>
       <c r="E466" s="3">
         <v>55</v>
       </c>
       <c r="F466" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.25">
@@ -27946,19 +28113,19 @@
         <v>1211</v>
       </c>
       <c r="B467" s="2" t="s">
-        <v>1225</v>
+        <v>1215</v>
       </c>
       <c r="C467" s="2" t="s">
-        <v>1221</v>
+        <v>1216</v>
       </c>
       <c r="D467" s="2" t="s">
-        <v>1226</v>
+        <v>1217</v>
       </c>
       <c r="E467" s="3">
         <v>55</v>
       </c>
       <c r="F467" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.25">
@@ -27966,19 +28133,19 @@
         <v>1211</v>
       </c>
       <c r="B468" s="2" t="s">
-        <v>1227</v>
+        <v>1218</v>
       </c>
       <c r="C468" s="2" t="s">
-        <v>1221</v>
+        <v>1213</v>
       </c>
       <c r="D468" s="2" t="s">
-        <v>1228</v>
+        <v>1219</v>
       </c>
       <c r="E468" s="3">
         <v>55</v>
       </c>
       <c r="F468" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.25">
@@ -27986,7 +28153,7 @@
         <v>1211</v>
       </c>
       <c r="B469" s="2" t="s">
-        <v>1229</v>
+        <v>1220</v>
       </c>
       <c r="C469" s="2" t="s">
         <v>1221</v>
@@ -27997,14 +28164,16 @@
       <c r="E469" s="3">
         <v>55</v>
       </c>
-      <c r="F469" s="2"/>
+      <c r="F469" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A470" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B470" s="2" t="s">
-        <v>1230</v>
+        <v>1223</v>
       </c>
       <c r="C470" s="2" t="s">
         <v>1221</v>
@@ -28015,14 +28184,16 @@
       <c r="E470" s="3">
         <v>55</v>
       </c>
-      <c r="F470" s="2"/>
+      <c r="F470" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A471" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B471" s="2" t="s">
-        <v>1231</v>
+        <v>1225</v>
       </c>
       <c r="C471" s="2" t="s">
         <v>1221</v>
@@ -28033,14 +28204,16 @@
       <c r="E471" s="3">
         <v>55</v>
       </c>
-      <c r="F471" s="2"/>
+      <c r="F471" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A472" s="2" t="s">
         <v>1211</v>
       </c>
       <c r="B472" s="2" t="s">
-        <v>1232</v>
+        <v>1227</v>
       </c>
       <c r="C472" s="2" t="s">
         <v>1221</v>
@@ -28051,7 +28224,9 @@
       <c r="E472" s="3">
         <v>55</v>
       </c>
-      <c r="F472" s="2"/>
+      <c r="F472" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A473" s="2" t="s">
@@ -28078,96 +28253,88 @@
         <v>1237</v>
       </c>
       <c r="B474" s="2" t="s">
-        <v>1238</v>
+        <v>1270</v>
       </c>
       <c r="C474" s="2" t="s">
-        <v>1239</v>
+        <v>1250</v>
       </c>
       <c r="D474" s="2" t="s">
-        <v>1240</v>
+        <v>1251</v>
       </c>
       <c r="E474" s="3">
-        <v>59</v>
-      </c>
-      <c r="F474" s="2" t="s">
-        <v>398</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="F474" s="2"/>
     </row>
     <row r="475" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A475" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B475" s="2" t="s">
-        <v>1241</v>
+        <v>1271</v>
       </c>
       <c r="C475" s="2" t="s">
-        <v>1239</v>
+        <v>1253</v>
       </c>
       <c r="D475" s="2" t="s">
-        <v>1242</v>
+        <v>1254</v>
       </c>
       <c r="E475" s="3">
-        <v>55</v>
-      </c>
-      <c r="F475" s="2" t="s">
-        <v>398</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="F475" s="2"/>
     </row>
     <row r="476" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A476" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B476" s="2" t="s">
-        <v>1243</v>
+        <v>1272</v>
       </c>
       <c r="C476" s="2" t="s">
-        <v>1239</v>
+        <v>1253</v>
       </c>
       <c r="D476" s="2" t="s">
-        <v>1244</v>
+        <v>1256</v>
       </c>
       <c r="E476" s="3">
         <v>55</v>
       </c>
-      <c r="F476" s="2" t="s">
-        <v>398</v>
-      </c>
+      <c r="F476" s="2"/>
     </row>
     <row r="477" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A477" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B477" s="2" t="s">
-        <v>1245</v>
+        <v>1273</v>
       </c>
       <c r="C477" s="2" t="s">
-        <v>1239</v>
+        <v>1253</v>
       </c>
       <c r="D477" s="2" t="s">
-        <v>1246</v>
+        <v>1258</v>
       </c>
       <c r="E477" s="3">
-        <v>75</v>
-      </c>
-      <c r="F477" s="2" t="s">
-        <v>398</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="F477" s="2"/>
     </row>
     <row r="478" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A478" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B478" s="2" t="s">
-        <v>1247</v>
+        <v>1238</v>
       </c>
       <c r="C478" s="2" t="s">
         <v>1239</v>
       </c>
       <c r="D478" s="2" t="s">
-        <v>1248</v>
+        <v>1240</v>
       </c>
       <c r="E478" s="3">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F478" s="2" t="s">
         <v>398</v>
@@ -28178,19 +28345,19 @@
         <v>1237</v>
       </c>
       <c r="B479" s="2" t="s">
-        <v>1249</v>
+        <v>1241</v>
       </c>
       <c r="C479" s="2" t="s">
-        <v>1250</v>
+        <v>1239</v>
       </c>
       <c r="D479" s="2" t="s">
-        <v>1251</v>
+        <v>1242</v>
       </c>
       <c r="E479" s="3">
         <v>55</v>
       </c>
       <c r="F479" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="480" spans="1:6" x14ac:dyDescent="0.25">
@@ -28198,19 +28365,19 @@
         <v>1237</v>
       </c>
       <c r="B480" s="2" t="s">
-        <v>1252</v>
+        <v>1243</v>
       </c>
       <c r="C480" s="2" t="s">
-        <v>1253</v>
+        <v>1239</v>
       </c>
       <c r="D480" s="2" t="s">
-        <v>1254</v>
+        <v>1244</v>
       </c>
       <c r="E480" s="3">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F480" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="481" spans="1:6" x14ac:dyDescent="0.25">
@@ -28218,19 +28385,19 @@
         <v>1237</v>
       </c>
       <c r="B481" s="2" t="s">
-        <v>1255</v>
+        <v>1245</v>
       </c>
       <c r="C481" s="2" t="s">
-        <v>1253</v>
+        <v>1239</v>
       </c>
       <c r="D481" s="2" t="s">
-        <v>1256</v>
+        <v>1246</v>
       </c>
       <c r="E481" s="3">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="F481" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="482" spans="1:6" x14ac:dyDescent="0.25">
@@ -28238,19 +28405,19 @@
         <v>1237</v>
       </c>
       <c r="B482" s="2" t="s">
-        <v>1257</v>
+        <v>1247</v>
       </c>
       <c r="C482" s="2" t="s">
-        <v>1253</v>
+        <v>1239</v>
       </c>
       <c r="D482" s="2" t="s">
-        <v>1258</v>
+        <v>1248</v>
       </c>
       <c r="E482" s="3">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F482" s="2" t="s">
-        <v>454</v>
+        <v>398</v>
       </c>
     </row>
     <row r="483" spans="1:6" x14ac:dyDescent="0.25">
@@ -28258,19 +28425,19 @@
         <v>1237</v>
       </c>
       <c r="B483" s="2" t="s">
-        <v>1259</v>
+        <v>1249</v>
       </c>
       <c r="C483" s="2" t="s">
-        <v>1260</v>
+        <v>1250</v>
       </c>
       <c r="D483" s="2" t="s">
-        <v>1261</v>
+        <v>1251</v>
       </c>
       <c r="E483" s="3">
         <v>55</v>
       </c>
       <c r="F483" s="2" t="s">
-        <v>491</v>
+        <v>454</v>
       </c>
     </row>
     <row r="484" spans="1:6" x14ac:dyDescent="0.25">
@@ -28278,19 +28445,19 @@
         <v>1237</v>
       </c>
       <c r="B484" s="2" t="s">
-        <v>1262</v>
+        <v>1252</v>
       </c>
       <c r="C484" s="2" t="s">
-        <v>1260</v>
+        <v>1253</v>
       </c>
       <c r="D484" s="2" t="s">
-        <v>1263</v>
+        <v>1254</v>
       </c>
       <c r="E484" s="3">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="F484" s="2" t="s">
-        <v>491</v>
+        <v>454</v>
       </c>
     </row>
     <row r="485" spans="1:6" x14ac:dyDescent="0.25">
@@ -28298,19 +28465,19 @@
         <v>1237</v>
       </c>
       <c r="B485" s="2" t="s">
-        <v>1274</v>
+        <v>1255</v>
       </c>
       <c r="C485" s="2" t="s">
-        <v>1275</v>
+        <v>1253</v>
       </c>
       <c r="D485" s="2" t="s">
-        <v>1276</v>
+        <v>1256</v>
       </c>
       <c r="E485" s="3">
         <v>55</v>
       </c>
       <c r="F485" s="2" t="s">
-        <v>10</v>
+        <v>454</v>
       </c>
     </row>
     <row r="486" spans="1:6" x14ac:dyDescent="0.25">
@@ -28318,19 +28485,19 @@
         <v>1237</v>
       </c>
       <c r="B486" s="2" t="s">
-        <v>1277</v>
+        <v>1257</v>
       </c>
       <c r="C486" s="2" t="s">
-        <v>1278</v>
+        <v>1253</v>
       </c>
       <c r="D486" s="2" t="s">
-        <v>1279</v>
+        <v>1258</v>
       </c>
       <c r="E486" s="3">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F486" s="2" t="s">
-        <v>10</v>
+        <v>454</v>
       </c>
     </row>
     <row r="487" spans="1:6" x14ac:dyDescent="0.25">
@@ -28338,126 +28505,140 @@
         <v>1237</v>
       </c>
       <c r="B487" s="2" t="s">
-        <v>1264</v>
+        <v>1259</v>
       </c>
       <c r="C487" s="2" t="s">
         <v>1260</v>
       </c>
       <c r="D487" s="2" t="s">
-        <v>1265</v>
+        <v>1261</v>
       </c>
       <c r="E487" s="3">
         <v>55</v>
       </c>
-      <c r="F487" s="2"/>
+      <c r="F487" s="2" t="s">
+        <v>491</v>
+      </c>
     </row>
     <row r="488" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A488" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B488" s="2" t="s">
-        <v>1266</v>
+        <v>1262</v>
       </c>
       <c r="C488" s="2" t="s">
         <v>1260</v>
       </c>
       <c r="D488" s="2" t="s">
-        <v>1267</v>
+        <v>1263</v>
       </c>
       <c r="E488" s="3">
-        <v>59</v>
-      </c>
-      <c r="F488" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="F488" s="2" t="s">
+        <v>491</v>
+      </c>
     </row>
     <row r="489" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A489" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B489" s="2" t="s">
-        <v>1268</v>
+        <v>1274</v>
       </c>
       <c r="C489" s="2" t="s">
-        <v>1260</v>
+        <v>1275</v>
       </c>
       <c r="D489" s="2" t="s">
-        <v>1269</v>
+        <v>1276</v>
       </c>
       <c r="E489" s="3">
         <v>55</v>
       </c>
-      <c r="F489" s="2"/>
+      <c r="F489" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="490" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A490" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B490" s="2" t="s">
-        <v>1270</v>
+        <v>1277</v>
       </c>
       <c r="C490" s="2" t="s">
-        <v>1250</v>
+        <v>1278</v>
       </c>
       <c r="D490" s="2" t="s">
-        <v>1251</v>
+        <v>1279</v>
       </c>
       <c r="E490" s="3">
         <v>55</v>
       </c>
-      <c r="F490" s="2"/>
+      <c r="F490" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="491" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A491" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B491" s="2" t="s">
-        <v>1271</v>
+        <v>1264</v>
       </c>
       <c r="C491" s="2" t="s">
-        <v>1253</v>
+        <v>1260</v>
       </c>
       <c r="D491" s="2" t="s">
-        <v>1254</v>
+        <v>1265</v>
       </c>
       <c r="E491" s="3">
-        <v>59</v>
-      </c>
-      <c r="F491" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="F491" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="492" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A492" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B492" s="2" t="s">
-        <v>1272</v>
+        <v>1266</v>
       </c>
       <c r="C492" s="2" t="s">
-        <v>1253</v>
+        <v>1260</v>
       </c>
       <c r="D492" s="2" t="s">
-        <v>1256</v>
+        <v>1267</v>
       </c>
       <c r="E492" s="3">
-        <v>55</v>
-      </c>
-      <c r="F492" s="2"/>
+        <v>59</v>
+      </c>
+      <c r="F492" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="493" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A493" s="2" t="s">
         <v>1237</v>
       </c>
       <c r="B493" s="2" t="s">
-        <v>1273</v>
+        <v>1268</v>
       </c>
       <c r="C493" s="2" t="s">
-        <v>1253</v>
+        <v>1260</v>
       </c>
       <c r="D493" s="2" t="s">
-        <v>1258</v>
+        <v>1269</v>
       </c>
       <c r="E493" s="3">
-        <v>59</v>
-      </c>
-      <c r="F493" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="F493" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="494" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A494" s="2" t="s">
@@ -28540,13 +28721,13 @@
         <v>1286</v>
       </c>
       <c r="B498" s="2" t="s">
-        <v>1293</v>
+        <v>1298</v>
       </c>
       <c r="C498" s="2" t="s">
-        <v>1294</v>
+        <v>1299</v>
       </c>
       <c r="D498" s="2" t="s">
-        <v>1295</v>
+        <v>856</v>
       </c>
       <c r="E498" s="3">
         <v>29</v>
@@ -28558,36 +28739,40 @@
         <v>1286</v>
       </c>
       <c r="B499" s="2" t="s">
-        <v>1296</v>
+        <v>1293</v>
       </c>
       <c r="C499" s="2" t="s">
         <v>1294</v>
       </c>
       <c r="D499" s="2" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
       <c r="E499" s="3">
         <v>29</v>
       </c>
-      <c r="F499" s="2"/>
+      <c r="F499" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="500" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A500" s="2" t="s">
         <v>1286</v>
       </c>
       <c r="B500" s="2" t="s">
-        <v>1298</v>
+        <v>1296</v>
       </c>
       <c r="C500" s="2" t="s">
-        <v>1299</v>
+        <v>1294</v>
       </c>
       <c r="D500" s="2" t="s">
-        <v>856</v>
+        <v>1297</v>
       </c>
       <c r="E500" s="3">
         <v>29</v>
       </c>
-      <c r="F500" s="2"/>
+      <c r="F500" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="501" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A501" s="2" t="s">
@@ -28743,7 +28928,9 @@
       <c r="E508" s="3">
         <v>100</v>
       </c>
-      <c r="F508" s="2"/>
+      <c r="F508" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="509" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A509" s="2" t="s">
@@ -28761,7 +28948,9 @@
       <c r="E509" s="3">
         <v>45</v>
       </c>
-      <c r="F509" s="2"/>
+      <c r="F509" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="510" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A510" s="2" t="s">
@@ -28935,7 +29124,9 @@
       <c r="E518" s="3">
         <v>66</v>
       </c>
-      <c r="F518" s="2"/>
+      <c r="F518" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="519" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A519" s="2" t="s">
@@ -29369,7 +29560,9 @@
       <c r="E540" s="3">
         <v>59</v>
       </c>
-      <c r="F540" s="2"/>
+      <c r="F540" s="2" t="s">
+        <v>6199</v>
+      </c>
     </row>
     <row r="541" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A541" s="2" t="s">
@@ -30521,7 +30714,9 @@
       <c r="E599" s="3">
         <v>45</v>
       </c>
-      <c r="F599" s="2"/>
+      <c r="F599" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="600" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A600" s="2" t="s">
@@ -30539,7 +30734,9 @@
       <c r="E600" s="3">
         <v>45</v>
       </c>
-      <c r="F600" s="2"/>
+      <c r="F600" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="601" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A601" s="2" t="s">
@@ -30667,7 +30864,9 @@
       <c r="E607" s="3">
         <v>50</v>
       </c>
-      <c r="F607" s="2"/>
+      <c r="F607" s="2" t="s">
+        <v>6215</v>
+      </c>
     </row>
     <row r="608" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A608" s="2" t="s">
@@ -30725,7 +30924,9 @@
       <c r="E610" s="3">
         <v>52</v>
       </c>
-      <c r="F610" s="2"/>
+      <c r="F610" s="2" t="s">
+        <v>6215</v>
+      </c>
     </row>
     <row r="611" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A611" s="2" t="s">
@@ -30743,45 +30944,47 @@
       <c r="E611" s="3">
         <v>52</v>
       </c>
-      <c r="F611" s="2"/>
+      <c r="F611" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="612" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A612" s="2" t="s">
         <v>1595</v>
       </c>
       <c r="B612" s="2" t="s">
-        <v>1596</v>
+        <v>1603</v>
       </c>
       <c r="C612" s="2" t="s">
-        <v>1597</v>
+        <v>1604</v>
       </c>
       <c r="D612" s="2" t="s">
-        <v>1598</v>
+        <v>1605</v>
       </c>
       <c r="E612" s="3">
         <v>60</v>
       </c>
-      <c r="F612" s="2"/>
+      <c r="F612" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="613" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A613" s="2" t="s">
         <v>1595</v>
       </c>
       <c r="B613" s="2" t="s">
-        <v>1603</v>
+        <v>1596</v>
       </c>
       <c r="C613" s="2" t="s">
-        <v>1604</v>
+        <v>1597</v>
       </c>
       <c r="D613" s="2" t="s">
-        <v>1605</v>
+        <v>1598</v>
       </c>
       <c r="E613" s="3">
         <v>60</v>
       </c>
-      <c r="F613" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F613" s="2"/>
     </row>
     <row r="614" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A614" s="2" t="s">
@@ -30835,7 +31038,9 @@
       <c r="E616" s="3">
         <v>50</v>
       </c>
-      <c r="F616" s="2"/>
+      <c r="F616" s="2" t="s">
+        <v>6215</v>
+      </c>
     </row>
     <row r="617" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A617" s="2" t="s">
@@ -30853,7 +31058,9 @@
       <c r="E617" s="3">
         <v>50</v>
       </c>
-      <c r="F617" s="2"/>
+      <c r="F617" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="618" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A618" s="2" t="s">
@@ -31037,7 +31244,9 @@
       <c r="E627" s="3">
         <v>35</v>
       </c>
-      <c r="F627" s="2"/>
+      <c r="F627" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="628" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A628" s="2" t="s">
@@ -31055,7 +31264,9 @@
       <c r="E628" s="3">
         <v>141</v>
       </c>
-      <c r="F628" s="2"/>
+      <c r="F628" s="2" t="s">
+        <v>6215</v>
+      </c>
     </row>
     <row r="629" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A629" s="2" t="s">
@@ -31073,7 +31284,9 @@
       <c r="E629" s="3">
         <v>141</v>
       </c>
-      <c r="F629" s="2"/>
+      <c r="F629" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="630" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A630" s="2" t="s">
@@ -31091,7 +31304,9 @@
       <c r="E630" s="3">
         <v>21</v>
       </c>
-      <c r="F630" s="2"/>
+      <c r="F630" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="631" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A631" s="2" t="s">
@@ -31249,7 +31464,9 @@
       <c r="E638" s="3">
         <v>176</v>
       </c>
-      <c r="F638" s="2"/>
+      <c r="F638" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="639" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A639" s="2" t="s">
@@ -31267,7 +31484,9 @@
       <c r="E639" s="3">
         <v>176</v>
       </c>
-      <c r="F639" s="2"/>
+      <c r="F639" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="640" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A640" s="2" t="s">
@@ -31285,7 +31504,9 @@
       <c r="E640" s="3">
         <v>176</v>
       </c>
-      <c r="F640" s="2"/>
+      <c r="F640" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="641" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A641" s="2" t="s">
@@ -31303,7 +31524,9 @@
       <c r="E641" s="3">
         <v>176</v>
       </c>
-      <c r="F641" s="2"/>
+      <c r="F641" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="642" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A642" s="2" t="s">
@@ -31321,7 +31544,9 @@
       <c r="E642" s="3">
         <v>176</v>
       </c>
-      <c r="F642" s="2"/>
+      <c r="F642" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="643" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A643" s="2" t="s">
@@ -31339,7 +31564,9 @@
       <c r="E643" s="3">
         <v>176</v>
       </c>
-      <c r="F643" s="2"/>
+      <c r="F643" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="644" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A644" s="2" t="s">
@@ -31357,7 +31584,9 @@
       <c r="E644" s="3">
         <v>176</v>
       </c>
-      <c r="F644" s="2"/>
+      <c r="F644" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="645" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A645" s="2" t="s">
@@ -31375,7 +31604,9 @@
       <c r="E645" s="3">
         <v>176</v>
       </c>
-      <c r="F645" s="2"/>
+      <c r="F645" s="2" t="s">
+        <v>6219</v>
+      </c>
     </row>
     <row r="646" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A646" s="2" t="s">
@@ -31519,7 +31750,9 @@
       <c r="E653" s="3">
         <v>115</v>
       </c>
-      <c r="F653" s="2"/>
+      <c r="F653" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="654" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A654" s="2" t="s">
@@ -31537,7 +31770,9 @@
       <c r="E654" s="3">
         <v>115</v>
       </c>
-      <c r="F654" s="2"/>
+      <c r="F654" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="655" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A655" s="2" t="s">
@@ -31555,7 +31790,9 @@
       <c r="E655" s="3">
         <v>115</v>
       </c>
-      <c r="F655" s="2"/>
+      <c r="F655" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="656" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A656" s="2" t="s">
@@ -31573,7 +31810,9 @@
       <c r="E656" s="3">
         <v>115</v>
       </c>
-      <c r="F656" s="2"/>
+      <c r="F656" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="657" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A657" s="2" t="s">
@@ -31591,7 +31830,9 @@
       <c r="E657" s="3">
         <v>95</v>
       </c>
-      <c r="F657" s="2"/>
+      <c r="F657" s="2" t="s">
+        <v>6216</v>
+      </c>
     </row>
     <row r="658" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A658" s="2" t="s">
@@ -31735,7 +31976,9 @@
       <c r="E665" s="3">
         <v>49</v>
       </c>
-      <c r="F665" s="2"/>
+      <c r="F665" s="2" t="s">
+        <v>6215</v>
+      </c>
     </row>
     <row r="666" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A666" s="2" t="s">
@@ -31753,7 +31996,9 @@
       <c r="E666" s="3">
         <v>49</v>
       </c>
-      <c r="F666" s="2"/>
+      <c r="F666" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="667" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A667" s="2" t="s">
@@ -32051,7 +32296,9 @@
       <c r="E681" s="3">
         <v>45</v>
       </c>
-      <c r="F681" s="2"/>
+      <c r="F681" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="682" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A682" s="2" t="s">
@@ -32069,7 +32316,9 @@
       <c r="E682" s="3">
         <v>45</v>
       </c>
-      <c r="F682" s="2"/>
+      <c r="F682" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="683" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A683" s="2" t="s">
@@ -32576,7 +32825,7 @@
         <v>1867</v>
       </c>
       <c r="B708" s="2" t="s">
-        <v>1868</v>
+        <v>1870</v>
       </c>
       <c r="C708" s="2" t="s">
         <v>1869</v>
@@ -32585,14 +32834,16 @@
       <c r="E708" s="3">
         <v>36</v>
       </c>
-      <c r="F708" s="2"/>
+      <c r="F708" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="709" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A709" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="B709" s="2" t="s">
-        <v>1870</v>
+        <v>1868</v>
       </c>
       <c r="C709" s="2" t="s">
         <v>1869</v>
@@ -32601,9 +32852,7 @@
       <c r="E709" s="3">
         <v>36</v>
       </c>
-      <c r="F709" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="F709" s="2"/>
     </row>
     <row r="710" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A710" s="2" t="s">
@@ -32777,7 +33026,9 @@
       <c r="E718" s="3">
         <v>43</v>
       </c>
-      <c r="F718" s="2"/>
+      <c r="F718" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="719" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A719" s="2" t="s">
@@ -32795,7 +33046,9 @@
       <c r="E719" s="3">
         <v>50</v>
       </c>
-      <c r="F719" s="2"/>
+      <c r="F719" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="720" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A720" s="2" t="s">
@@ -32813,7 +33066,9 @@
       <c r="E720" s="3">
         <v>50</v>
       </c>
-      <c r="F720" s="2"/>
+      <c r="F720" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="721" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A721" s="2" t="s">
@@ -32831,7 +33086,9 @@
       <c r="E721" s="3">
         <v>48</v>
       </c>
-      <c r="F721" s="2"/>
+      <c r="F721" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="722" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A722" s="2" t="s">
@@ -32849,7 +33106,9 @@
       <c r="E722" s="3">
         <v>48</v>
       </c>
-      <c r="F722" s="2"/>
+      <c r="F722" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="723" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A723" s="2" t="s">
@@ -33853,7 +34112,9 @@
       <c r="E773" s="3">
         <v>32</v>
       </c>
-      <c r="F773" s="2"/>
+      <c r="F773" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="774" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A774" s="2" t="s">
@@ -33871,7 +34132,9 @@
       <c r="E774" s="3">
         <v>32</v>
       </c>
-      <c r="F774" s="2"/>
+      <c r="F774" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="775" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A775" s="2" t="s">
@@ -34207,7 +34470,9 @@
       <c r="E791" s="3">
         <v>55</v>
       </c>
-      <c r="F791" s="2"/>
+      <c r="F791" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="792" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A792" s="2" t="s">
@@ -34225,7 +34490,9 @@
       <c r="E792" s="3">
         <v>55</v>
       </c>
-      <c r="F792" s="2"/>
+      <c r="F792" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="793" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A793" s="2" t="s">
@@ -34243,7 +34510,9 @@
       <c r="E793" s="3">
         <v>55</v>
       </c>
-      <c r="F793" s="2"/>
+      <c r="F793" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="794" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A794" s="2" t="s">
@@ -34261,7 +34530,9 @@
       <c r="E794" s="3">
         <v>55</v>
       </c>
-      <c r="F794" s="2"/>
+      <c r="F794" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="795" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A795" s="2" t="s">
@@ -34359,7 +34630,9 @@
       <c r="E799" s="3">
         <v>38</v>
       </c>
-      <c r="F799" s="2"/>
+      <c r="F799" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="800" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A800" s="2" t="s">
@@ -34377,7 +34650,9 @@
       <c r="E800" s="3">
         <v>38</v>
       </c>
-      <c r="F800" s="2"/>
+      <c r="F800" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="801" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A801" s="2" t="s">
@@ -34395,7 +34670,9 @@
       <c r="E801" s="3">
         <v>38</v>
       </c>
-      <c r="F801" s="2"/>
+      <c r="F801" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="802" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A802" s="2" t="s">
@@ -34413,7 +34690,9 @@
       <c r="E802" s="3">
         <v>38</v>
       </c>
-      <c r="F802" s="2"/>
+      <c r="F802" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="803" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A803" s="2" t="s">
@@ -34431,7 +34710,9 @@
       <c r="E803" s="3">
         <v>35</v>
       </c>
-      <c r="F803" s="2"/>
+      <c r="F803" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="804" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A804" s="2" t="s">
@@ -34449,7 +34730,9 @@
       <c r="E804" s="3">
         <v>35</v>
       </c>
-      <c r="F804" s="2"/>
+      <c r="F804" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="805" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A805" s="2" t="s">
@@ -34467,7 +34750,9 @@
       <c r="E805" s="3">
         <v>35</v>
       </c>
-      <c r="F805" s="2"/>
+      <c r="F805" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="806" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A806" s="2" t="s">
@@ -34485,7 +34770,9 @@
       <c r="E806" s="3">
         <v>35</v>
       </c>
-      <c r="F806" s="2"/>
+      <c r="F806" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="807" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A807" s="2" t="s">
@@ -34583,7 +34870,9 @@
       <c r="E811" s="3">
         <v>47</v>
       </c>
-      <c r="F811" s="2"/>
+      <c r="F811" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="812" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A812" s="2" t="s">
@@ -34601,7 +34890,9 @@
       <c r="E812" s="3">
         <v>47</v>
       </c>
-      <c r="F812" s="2"/>
+      <c r="F812" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="813" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A813" s="2" t="s">
@@ -34619,7 +34910,9 @@
       <c r="E813" s="3">
         <v>47</v>
       </c>
-      <c r="F813" s="2"/>
+      <c r="F813" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="814" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A814" s="2" t="s">
@@ -34637,7 +34930,9 @@
       <c r="E814" s="3">
         <v>47</v>
       </c>
-      <c r="F814" s="2"/>
+      <c r="F814" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="815" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A815" s="2" t="s">
@@ -34655,7 +34950,9 @@
       <c r="E815" s="3">
         <v>47</v>
       </c>
-      <c r="F815" s="2"/>
+      <c r="F815" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="816" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A816" s="2" t="s">
@@ -34673,7 +34970,9 @@
       <c r="E816" s="3">
         <v>47</v>
       </c>
-      <c r="F816" s="2"/>
+      <c r="F816" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="817" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A817" s="2" t="s">
@@ -34691,7 +34990,9 @@
       <c r="E817" s="3">
         <v>47</v>
       </c>
-      <c r="F817" s="2"/>
+      <c r="F817" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="818" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A818" s="2" t="s">
@@ -34709,7 +35010,9 @@
       <c r="E818" s="3">
         <v>47</v>
       </c>
-      <c r="F818" s="2"/>
+      <c r="F818" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="819" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A819" s="2" t="s">
@@ -34767,7 +35070,9 @@
       <c r="E821" s="3">
         <v>50</v>
       </c>
-      <c r="F821" s="2"/>
+      <c r="F821" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="822" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A822" s="2" t="s">
@@ -34785,7 +35090,9 @@
       <c r="E822" s="3">
         <v>50</v>
       </c>
-      <c r="F822" s="2"/>
+      <c r="F822" s="2" t="s">
+        <v>6214</v>
+      </c>
     </row>
     <row r="823" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A823" s="2" t="s">
@@ -38901,7 +39208,9 @@
       <c r="E1032" s="3">
         <v>28</v>
       </c>
-      <c r="F1032" s="2"/>
+      <c r="F1032" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="1033" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1033" s="2" t="s">
@@ -38919,7 +39228,9 @@
       <c r="E1033" s="3">
         <v>28</v>
       </c>
-      <c r="F1033" s="2"/>
+      <c r="F1033" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="1034" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1034" s="2" t="s">
@@ -38937,7 +39248,9 @@
       <c r="E1034" s="3">
         <v>85</v>
       </c>
-      <c r="F1034" s="2"/>
+      <c r="F1034" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1035" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1035" s="2" t="s">
@@ -38955,7 +39268,9 @@
       <c r="E1035" s="3">
         <v>85</v>
       </c>
-      <c r="F1035" s="2"/>
+      <c r="F1035" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1036" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1036" s="2" t="s">
@@ -38973,7 +39288,9 @@
       <c r="E1036" s="3">
         <v>85</v>
       </c>
-      <c r="F1036" s="2"/>
+      <c r="F1036" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1037" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1037" s="2" t="s">
@@ -38991,7 +39308,9 @@
       <c r="E1037" s="3">
         <v>85</v>
       </c>
-      <c r="F1037" s="2"/>
+      <c r="F1037" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1038" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1038" s="2" t="s">
@@ -39009,7 +39328,9 @@
       <c r="E1038" s="3">
         <v>85</v>
       </c>
-      <c r="F1038" s="2"/>
+      <c r="F1038" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1039" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1039" s="2" t="s">
@@ -39027,7 +39348,9 @@
       <c r="E1039" s="3">
         <v>85</v>
       </c>
-      <c r="F1039" s="2"/>
+      <c r="F1039" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1040" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1040" s="2" t="s">
@@ -39045,7 +39368,9 @@
       <c r="E1040" s="3">
         <v>85</v>
       </c>
-      <c r="F1040" s="2"/>
+      <c r="F1040" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1041" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1041" s="2" t="s">
@@ -39063,7 +39388,9 @@
       <c r="E1041" s="3">
         <v>85</v>
       </c>
-      <c r="F1041" s="2"/>
+      <c r="F1041" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1042" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1042" s="2" t="s">
@@ -39081,7 +39408,9 @@
       <c r="E1042" s="3">
         <v>85</v>
       </c>
-      <c r="F1042" s="2"/>
+      <c r="F1042" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1043" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1043" s="2" t="s">
@@ -39099,7 +39428,9 @@
       <c r="E1043" s="3">
         <v>85</v>
       </c>
-      <c r="F1043" s="2"/>
+      <c r="F1043" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1044" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1044" s="2" t="s">
@@ -39117,7 +39448,9 @@
       <c r="E1044" s="3">
         <v>85</v>
       </c>
-      <c r="F1044" s="2"/>
+      <c r="F1044" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1045" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1045" s="2" t="s">
@@ -39135,7 +39468,9 @@
       <c r="E1045" s="3">
         <v>85</v>
       </c>
-      <c r="F1045" s="2"/>
+      <c r="F1045" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1046" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1046" s="2" t="s">
@@ -39153,7 +39488,9 @@
       <c r="E1046" s="3">
         <v>35</v>
       </c>
-      <c r="F1046" s="2"/>
+      <c r="F1046" s="2" t="s">
+        <v>6213</v>
+      </c>
     </row>
     <row r="1047" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1047" s="2" t="s">
@@ -39315,7 +39652,9 @@
       <c r="E1055" s="3">
         <v>36</v>
       </c>
-      <c r="F1055" s="2"/>
+      <c r="F1055" s="2" t="s">
+        <v>6218</v>
+      </c>
     </row>
     <row r="1056" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1056" s="2" t="s">
@@ -39331,7 +39670,9 @@
       <c r="E1056" s="3">
         <v>55</v>
       </c>
-      <c r="F1056" s="2"/>
+      <c r="F1056" s="2" t="s">
+        <v>6218</v>
+      </c>
     </row>
     <row r="1057" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1057" s="2" t="s">
@@ -39347,7 +39688,9 @@
       <c r="E1057" s="3">
         <v>55</v>
       </c>
-      <c r="F1057" s="2"/>
+      <c r="F1057" s="2" t="s">
+        <v>6218</v>
+      </c>
     </row>
     <row r="1058" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1058" s="2" t="s">
@@ -39363,7 +39706,9 @@
       <c r="E1058" s="3">
         <v>39</v>
       </c>
-      <c r="F1058" s="2"/>
+      <c r="F1058" s="2" t="s">
+        <v>6218</v>
+      </c>
     </row>
     <row r="1059" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1059" s="2" t="s">
@@ -39517,7 +39862,9 @@
       <c r="E1066" s="3">
         <v>32</v>
       </c>
-      <c r="F1066" s="2"/>
+      <c r="F1066" s="2" t="s">
+        <v>6217</v>
+      </c>
     </row>
     <row r="1067" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1067" s="2" t="s">
@@ -39533,7 +39880,9 @@
       <c r="E1067" s="3">
         <v>32</v>
       </c>
-      <c r="F1067" s="2"/>
+      <c r="F1067" s="2" t="s">
+        <v>6217</v>
+      </c>
     </row>
     <row r="1068" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1068" s="2" t="s">
@@ -40829,7 +41178,9 @@
       <c r="E1134" s="3">
         <v>85</v>
       </c>
-      <c r="F1134" s="2"/>
+      <c r="F1134" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1135" s="2" t="s">
@@ -40847,7 +41198,9 @@
       <c r="E1135" s="3">
         <v>85</v>
       </c>
-      <c r="F1135" s="2"/>
+      <c r="F1135" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1136" s="2" t="s">
@@ -40865,7 +41218,9 @@
       <c r="E1136" s="3">
         <v>85</v>
       </c>
-      <c r="F1136" s="2"/>
+      <c r="F1136" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1137" s="2" t="s">
@@ -40883,7 +41238,9 @@
       <c r="E1137" s="3">
         <v>85</v>
       </c>
-      <c r="F1137" s="2"/>
+      <c r="F1137" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1138" s="2" t="s">
@@ -40901,7 +41258,9 @@
       <c r="E1138" s="3">
         <v>85</v>
       </c>
-      <c r="F1138" s="2"/>
+      <c r="F1138" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1139" s="2" t="s">
@@ -40919,7 +41278,9 @@
       <c r="E1139" s="3">
         <v>85</v>
       </c>
-      <c r="F1139" s="2"/>
+      <c r="F1139" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1140" s="2" t="s">
@@ -40937,7 +41298,9 @@
       <c r="E1140" s="3">
         <v>85</v>
       </c>
-      <c r="F1140" s="2"/>
+      <c r="F1140" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1141" s="2" t="s">
@@ -40955,7 +41318,9 @@
       <c r="E1141" s="3">
         <v>85</v>
       </c>
-      <c r="F1141" s="2"/>
+      <c r="F1141" s="2" t="s">
+        <v>6212</v>
+      </c>
     </row>
     <row r="1142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1142" s="2" t="s">
@@ -41693,7 +42058,9 @@
       <c r="E1178" s="3">
         <v>45</v>
       </c>
-      <c r="F1178" s="2"/>
+      <c r="F1178" s="2" t="s">
+        <v>6200</v>
+      </c>
     </row>
     <row r="1179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1179" s="2" t="s">
@@ -41711,7 +42078,9 @@
       <c r="E1179" s="3">
         <v>45</v>
       </c>
-      <c r="F1179" s="2"/>
+      <c r="F1179" s="2" t="s">
+        <v>6200</v>
+      </c>
     </row>
     <row r="1180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1180" s="2" t="s">
@@ -41729,7 +42098,9 @@
       <c r="E1180" s="3">
         <v>45</v>
       </c>
-      <c r="F1180" s="2"/>
+      <c r="F1180" s="2" t="s">
+        <v>6200</v>
+      </c>
     </row>
     <row r="1181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1181" s="2" t="s">
@@ -41747,7 +42118,9 @@
       <c r="E1181" s="3">
         <v>45</v>
       </c>
-      <c r="F1181" s="2"/>
+      <c r="F1181" s="2" t="s">
+        <v>6200</v>
+      </c>
     </row>
     <row r="1182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1182" s="2" t="s">
@@ -41965,7 +42338,9 @@
       <c r="E1192" s="3">
         <v>55</v>
       </c>
-      <c r="F1192" s="2"/>
+      <c r="F1192" s="2" t="s">
+        <v>6211</v>
+      </c>
     </row>
     <row r="1193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1193" s="2" t="s">
@@ -41983,7 +42358,9 @@
       <c r="E1193" s="3">
         <v>55</v>
       </c>
-      <c r="F1193" s="2"/>
+      <c r="F1193" s="2" t="s">
+        <v>6211</v>
+      </c>
     </row>
     <row r="1194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1194" s="2" t="s">
@@ -44681,7 +45058,9 @@
       <c r="E1330" s="3">
         <v>40</v>
       </c>
-      <c r="F1330" s="2"/>
+      <c r="F1330" s="2" t="s">
+        <v>6210</v>
+      </c>
     </row>
     <row r="1331" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1331" s="2" t="s">
@@ -44699,7 +45078,9 @@
       <c r="E1331" s="3">
         <v>40</v>
       </c>
-      <c r="F1331" s="2"/>
+      <c r="F1331" s="2" t="s">
+        <v>6210</v>
+      </c>
     </row>
     <row r="1332" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1332" s="2" t="s">
@@ -45437,7 +45818,9 @@
       <c r="E1368" s="3">
         <v>70</v>
       </c>
-      <c r="F1368" s="2"/>
+      <c r="F1368" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1369" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1369" s="2" t="s">
@@ -45455,7 +45838,9 @@
       <c r="E1369" s="3">
         <v>70</v>
       </c>
-      <c r="F1369" s="2"/>
+      <c r="F1369" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1370" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1370" s="2" t="s">
@@ -45473,7 +45858,9 @@
       <c r="E1370" s="3">
         <v>70</v>
       </c>
-      <c r="F1370" s="2"/>
+      <c r="F1370" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1371" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1371" s="2" t="s">
@@ -45491,7 +45878,9 @@
       <c r="E1371" s="3">
         <v>70</v>
       </c>
-      <c r="F1371" s="2"/>
+      <c r="F1371" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1372" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1372" s="2" t="s">
@@ -45509,7 +45898,9 @@
       <c r="E1372" s="3">
         <v>70</v>
       </c>
-      <c r="F1372" s="2"/>
+      <c r="F1372" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1373" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1373" s="2" t="s">
@@ -45527,7 +45918,9 @@
       <c r="E1373" s="3">
         <v>70</v>
       </c>
-      <c r="F1373" s="2"/>
+      <c r="F1373" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1374" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1374" s="2" t="s">
@@ -45545,7 +45938,9 @@
       <c r="E1374" s="3">
         <v>70</v>
       </c>
-      <c r="F1374" s="2"/>
+      <c r="F1374" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1375" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1375" s="2" t="s">
@@ -45563,7 +45958,9 @@
       <c r="E1375" s="3">
         <v>70</v>
       </c>
-      <c r="F1375" s="2"/>
+      <c r="F1375" s="2" t="s">
+        <v>6209</v>
+      </c>
     </row>
     <row r="1376" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1376" s="2" t="s">
@@ -46721,7 +47118,9 @@
       <c r="E1433" s="3">
         <v>25</v>
       </c>
-      <c r="F1433" s="2"/>
+      <c r="F1433" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="1434" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1434" s="2" t="s">
@@ -46739,7 +47138,9 @@
       <c r="E1434" s="3">
         <v>11</v>
       </c>
-      <c r="F1434" s="2"/>
+      <c r="F1434" s="2" t="s">
+        <v>6202</v>
+      </c>
     </row>
     <row r="1435" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1435" s="2" t="s">
@@ -47411,7 +47812,9 @@
       <c r="E1468" s="3">
         <v>36</v>
       </c>
-      <c r="F1468" s="2"/>
+      <c r="F1468" s="2" t="s">
+        <v>6208</v>
+      </c>
     </row>
     <row r="1469" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1469" s="2" t="s">
@@ -47427,7 +47830,9 @@
       <c r="E1469" s="3">
         <v>36</v>
       </c>
-      <c r="F1469" s="2"/>
+      <c r="F1469" s="2" t="s">
+        <v>6208</v>
+      </c>
     </row>
     <row r="1470" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1470" s="2" t="s">
@@ -48757,7 +49162,9 @@
       <c r="E1536" s="3">
         <v>35</v>
       </c>
-      <c r="F1536" s="2"/>
+      <c r="F1536" s="2" t="s">
+        <v>6207</v>
+      </c>
     </row>
     <row r="1537" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1537" s="2" t="s">
@@ -48991,7 +49398,9 @@
       <c r="E1548" s="3">
         <v>35</v>
       </c>
-      <c r="F1548" s="2"/>
+      <c r="F1548" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1549" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1549" s="2" t="s">
@@ -49009,7 +49418,9 @@
       <c r="E1549" s="3">
         <v>35</v>
       </c>
-      <c r="F1549" s="2"/>
+      <c r="F1549" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1550" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1550" s="2" t="s">
@@ -49027,7 +49438,9 @@
       <c r="E1550" s="3">
         <v>35</v>
       </c>
-      <c r="F1550" s="2"/>
+      <c r="F1550" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1551" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1551" s="2" t="s">
@@ -51761,7 +52174,9 @@
       <c r="E1687" s="3">
         <v>80</v>
       </c>
-      <c r="F1687" s="2"/>
+      <c r="F1687" s="2" t="s">
+        <v>6206</v>
+      </c>
     </row>
     <row r="1688" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1688" s="2" t="s">
@@ -51779,7 +52194,9 @@
       <c r="E1688" s="3">
         <v>90</v>
       </c>
-      <c r="F1688" s="2"/>
+      <c r="F1688" s="2" t="s">
+        <v>6206</v>
+      </c>
     </row>
     <row r="1689" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1689" s="2" t="s">
@@ -51797,7 +52214,9 @@
       <c r="E1689" s="3">
         <v>55</v>
       </c>
-      <c r="F1689" s="2"/>
+      <c r="F1689" s="2" t="s">
+        <v>6206</v>
+      </c>
     </row>
     <row r="1690" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1690" s="2" t="s">
@@ -51815,7 +52234,9 @@
       <c r="E1690" s="3">
         <v>55</v>
       </c>
-      <c r="F1690" s="2"/>
+      <c r="F1690" s="2" t="s">
+        <v>6206</v>
+      </c>
     </row>
     <row r="1691" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1691" s="2" t="s">
@@ -51833,7 +52254,9 @@
       <c r="E1691" s="3">
         <v>33</v>
       </c>
-      <c r="F1691" s="2"/>
+      <c r="F1691" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1692" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1692" s="2" t="s">
@@ -51851,7 +52274,9 @@
       <c r="E1692" s="3">
         <v>54</v>
       </c>
-      <c r="F1692" s="2"/>
+      <c r="F1692" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1693" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1693" s="2" t="s">
@@ -51869,7 +52294,9 @@
       <c r="E1693" s="3">
         <v>130</v>
       </c>
-      <c r="F1693" s="2"/>
+      <c r="F1693" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1694" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1694" s="2" t="s">
@@ -51887,7 +52314,9 @@
       <c r="E1694" s="3">
         <v>130</v>
       </c>
-      <c r="F1694" s="2"/>
+      <c r="F1694" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1695" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1695" s="2" t="s">
@@ -51905,7 +52334,9 @@
       <c r="E1695" s="3">
         <v>37</v>
       </c>
-      <c r="F1695" s="2"/>
+      <c r="F1695" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1696" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1696" s="2" t="s">
@@ -51923,7 +52354,9 @@
       <c r="E1696" s="3">
         <v>37</v>
       </c>
-      <c r="F1696" s="2"/>
+      <c r="F1696" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1697" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1697" s="2" t="s">
@@ -53619,7 +54052,9 @@
       <c r="E1782" s="3">
         <v>118</v>
       </c>
-      <c r="F1782" s="2"/>
+      <c r="F1782" s="2" t="s">
+        <v>6205</v>
+      </c>
     </row>
     <row r="1783" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1783" s="2" t="s">
@@ -53635,7 +54070,9 @@
       <c r="E1783" s="3">
         <v>118</v>
       </c>
-      <c r="F1783" s="2"/>
+      <c r="F1783" s="2" t="s">
+        <v>6205</v>
+      </c>
     </row>
     <row r="1784" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1784" s="2" t="s">
@@ -53653,7 +54090,9 @@
       <c r="E1784" s="3">
         <v>50</v>
       </c>
-      <c r="F1784" s="2"/>
+      <c r="F1784" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1785" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1785" s="2" t="s">
@@ -53671,7 +54110,9 @@
       <c r="E1785" s="3">
         <v>55</v>
       </c>
-      <c r="F1785" s="2"/>
+      <c r="F1785" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1786" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1786" s="2" t="s">
@@ -53749,7 +54190,9 @@
       <c r="E1789" s="3">
         <v>50</v>
       </c>
-      <c r="F1789" s="2"/>
+      <c r="F1789" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1790" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1790" s="2" t="s">
@@ -53767,7 +54210,9 @@
       <c r="E1790" s="3">
         <v>55</v>
       </c>
-      <c r="F1790" s="2"/>
+      <c r="F1790" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1791" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1791" s="2" t="s">
@@ -53785,7 +54230,9 @@
       <c r="E1791" s="3">
         <v>65</v>
       </c>
-      <c r="F1791" s="2"/>
+      <c r="F1791" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1792" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1792" s="2" t="s">
@@ -53803,7 +54250,9 @@
       <c r="E1792" s="3">
         <v>65</v>
       </c>
-      <c r="F1792" s="2"/>
+      <c r="F1792" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1793" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1793" s="2" t="s">
@@ -53821,7 +54270,9 @@
       <c r="E1793" s="3">
         <v>50</v>
       </c>
-      <c r="F1793" s="2"/>
+      <c r="F1793" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1794" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1794" s="2" t="s">
@@ -53839,7 +54290,9 @@
       <c r="E1794" s="3">
         <v>50</v>
       </c>
-      <c r="F1794" s="2"/>
+      <c r="F1794" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1795" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1795" s="2" t="s">
@@ -53857,7 +54310,9 @@
       <c r="E1795" s="3">
         <v>65</v>
       </c>
-      <c r="F1795" s="2"/>
+      <c r="F1795" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1796" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1796" s="2" t="s">
@@ -53875,7 +54330,9 @@
       <c r="E1796" s="3">
         <v>65</v>
       </c>
-      <c r="F1796" s="2"/>
+      <c r="F1796" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1797" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1797" s="2" t="s">
@@ -53893,7 +54350,9 @@
       <c r="E1797" s="3">
         <v>65</v>
       </c>
-      <c r="F1797" s="2"/>
+      <c r="F1797" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1798" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1798" s="2" t="s">
@@ -53911,7 +54370,9 @@
       <c r="E1798" s="3">
         <v>65</v>
       </c>
-      <c r="F1798" s="2"/>
+      <c r="F1798" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1799" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1799" s="2" t="s">
@@ -53929,7 +54390,9 @@
       <c r="E1799" s="3">
         <v>55</v>
       </c>
-      <c r="F1799" s="2"/>
+      <c r="F1799" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1800" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1800" s="2" t="s">
@@ -53947,7 +54410,9 @@
       <c r="E1800" s="3">
         <v>55</v>
       </c>
-      <c r="F1800" s="2"/>
+      <c r="F1800" s="2" t="s">
+        <v>6204</v>
+      </c>
     </row>
     <row r="1801" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1801" s="2" t="s">
@@ -56127,7 +56592,9 @@
       <c r="E1910" s="3">
         <v>65</v>
       </c>
-      <c r="F1910" s="2"/>
+      <c r="F1910" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1911" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1911" s="2" t="s">
@@ -56145,7 +56612,9 @@
       <c r="E1911" s="3">
         <v>65</v>
       </c>
-      <c r="F1911" s="2"/>
+      <c r="F1911" s="2" t="s">
+        <v>6203</v>
+      </c>
     </row>
     <row r="1912" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1912" s="2" t="s">
@@ -57001,7 +57470,9 @@
       <c r="E1954" s="3">
         <v>65</v>
       </c>
-      <c r="F1954" s="2"/>
+      <c r="F1954" s="2" t="s">
+        <v>6201</v>
+      </c>
     </row>
     <row r="1955" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1955" s="2" t="s">
@@ -57019,7 +57490,9 @@
       <c r="E1955" s="3">
         <v>57</v>
       </c>
-      <c r="F1955" s="2"/>
+      <c r="F1955" s="2" t="s">
+        <v>6201</v>
+      </c>
     </row>
     <row r="1956" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1956" s="2" t="s">
@@ -57037,7 +57510,9 @@
       <c r="E1956" s="3">
         <v>51</v>
       </c>
-      <c r="F1956" s="2"/>
+      <c r="F1956" s="2" t="s">
+        <v>6201</v>
+      </c>
     </row>
     <row r="1957" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1957" s="2" t="s">
@@ -57053,7 +57528,9 @@
       <c r="E1957" s="3">
         <v>55</v>
       </c>
-      <c r="F1957" s="2"/>
+      <c r="F1957" s="2" t="s">
+        <v>6201</v>
+      </c>
     </row>
     <row r="1958" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1958" s="2" t="s">
@@ -57069,7 +57546,9 @@
       <c r="E1958" s="3">
         <v>55</v>
       </c>
-      <c r="F1958" s="2"/>
+      <c r="F1958" s="2" t="s">
+        <v>6201</v>
+      </c>
     </row>
     <row r="1959" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1959" s="2" t="s">
@@ -59397,7 +59876,9 @@
       <c r="E2075" s="3">
         <v>35</v>
       </c>
-      <c r="F2075" s="2"/>
+      <c r="F2075" s="2" t="s">
+        <v>6200</v>
+      </c>
     </row>
     <row r="2076" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2076" s="2" t="s">
@@ -59415,7 +59896,9 @@
       <c r="E2076" s="3">
         <v>35</v>
       </c>
-      <c r="F2076" s="2"/>
+      <c r="F2076" s="2" t="s">
+        <v>6200</v>
+      </c>
     </row>
     <row r="2077" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2077" s="2" t="s">

</xml_diff>